<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.001-04 Le bateau de Mila
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-04.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-04.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila veut le bateau bleu du port. Le doudou est dans le manteau, le loquet résiste. Elle pousse, range, pose le pied sur le bois.</t>
+          <t>Sous le plancher, le bois du quai tape. Un éclat de corde pâle brille sur le rebord. Mila veut porter son dessin jusqu'au bateau bleu, maintenant. Elle pousse tout dans le sac : le zip mord, le bateau jaune se plie. Maman s'accroupit. Une chose, puis la suivante. Un souffle glisse le dessin vers la fenêtre. Mila refuse de foncer. L'éclat de corde penche : c'est le vent. Elle ferme, glisse l'éclat, puis le dessin. Sur le bois du bateau, l'éclat porte une trace de sel.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>L'eau du port claque contre le bois. Une corde mouillée sent le sel. Les mâts bougent un tout petit peu. Dans l'appartement au-dessus du quai, ça sent le savon. Une mouette crie, tout près de la vitre. Le dessin de Mila sèche près de la fenêtre. Il sent encore un peu la peinture. Un bateau bleu attend au bout du quai. Mila, tu entends l'eau ? Oui, maman. Je veux le bateau. On y va, avec le sac. En ce moment, Mila touche la sangle. Maman pose le sac bleu près des chaussures. Le tissu est un peu rêche. Une chaussure rouge est là. L'autre n'est pas là. Il est bleu, maman. Oui, prends de l'eau pour le quai. Mila prend la gourde. Elle est froide contre ses doigts. Elle la met dans le sac. Le goûter sent la pomme. Le papier fait un petit bruit. Glisse aussi le goûter. Mila le glisse près de l'eau. Et mon doudou ? Le doudou n'est pas près des chaussures. Regarde dans la poche du manteau. Mila cherche dans la poche. Le doudou sent le coton. Il était caché. Elle le glisse dans le sac. On ouvre ? Le loquet de la porte résiste. Il reste, maman. Pousse le petit bouton, tout doux.</t>
+          <t>Sous le plancher, le bois du quai tape. Le son grimpe l'escalier, puis la pièce. Dans l'appartement, ça sent le savon et le sel. Une mouette crie contre la vitre. Sur le rebord, un éclat de corde brille. Il est pâle, raide, et il sent le sel. Le vent du port l'a posé là. Mila ne sait pas à quoi il servira. Son dessin du bateau sèche sur la table. La peinture jaune luit, un peu collante. En bas, le vrai bateau bleu frappe le quai. Je veux le bateau, maintenant ! Mila, tu entends l'eau ? Oui, maman. Il m'attend. On y va, avec le sac. En ce moment, Mila saisit le sac bleu. Le tissu gratte sous ses doigts. La sangle sent le sel, comme la corde. Prends de l'eau, pour le quai. Mila prend la gourde froide. Le goûter sent la pomme, dans son papier. Je mets tout, d'un coup ! Elle pousse gourde, pomme et dessin. Le zip mord le papier du dessin. Le bateau jaune se plie, de travers. Ça reste coincé ! Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>L'eau du port claque contre le bois. Une corde mouillée sent le sel. Les mâts bougent un tout petit peu. Dans l'appartement au-dessus du quai, ça sent le savon. Une mouette crie, tout près de la vitre. Le dessin de Mila sèche près de la fenêtre. Il sent encore un peu la peinture. Un bateau bleu attend au bout du quai. Mila, tu entends l'eau ? Oui, maman. Je veux le bateau. On y va, avec le sac. En ce moment, Mila touche la sangle. Maman pose le sac bleu près des chaussures. Le tissu est un peu rêche. Une chaussure rouge est là. L'autre n'est pas là. Il est bleu, maman. Oui, prends de l'eau pour le quai. Mila prend la gourde. Elle est froide contre ses doigts. Elle la met dans le sac. Le goûter sent la pomme. Le papier fait un petit bruit. Glisse aussi le goûter. Mila le glisse près de l'eau. Et mon doudou ? Le doudou n'est pas près des chaussures. Regarde dans la poche du manteau. Mila cherche dans la poche. Le doudou sent le coton. Il était caché. Elle le glisse dans le sac. On ouvre ? Le loquet de la porte résiste. Il reste, maman. Pousse le petit bouton, tout doux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sous le plancher, le bois du quai tape. Le son grimpe l'escalier, puis la pièce. Dans l'appartement, ça sent le savon et le sel. Une mouette crie contre la vitre. Sur le rebord, un &lt;emphasis level="moderate"&gt;éclat de corde&lt;/emphasis&gt; brille. Il est pâle, raide, et il sent le sel. Le vent du port l'a posé là. Mila ne sait pas à quoi il servira. Son dessin du bateau sèche sur la table. La peinture jaune luit, un peu collante. En bas, le vrai bateau bleu frappe le quai. Je veux le bateau, maintenant ! Mila, tu entends l'eau ? Oui, maman. Il m'attend. On y va, avec le sac. En ce moment, Mila saisit le sac bleu. Le tissu gratte sous ses doigts. La sangle sent le sel, comme la corde. Prends de l'eau, pour le quai. Mila prend la gourde froide. Le goûter sent la pomme, dans son papier. Je mets tout, d'un coup ! Elle pousse gourde, pomme et dessin. Le zip mord le papier du dessin. Le bateau jaune se plie, de travers. Ça reste coincé ! Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Léa est dans l'entrée. Maman pose le &lt;emphasis&gt;sac&lt;/emphasis&gt; bleu. Maman dit : on met dans le sac ce que l'adulte a dit. L'adulte, c'est maman. Maman a dit : la gourde, le goûter, le doudou. Léa met la gourde. Elle met le goûter. Elle glisse le doudou. Elle ferme le zip. Maman dit : c'est ce que l'adulte a dit. Léa répète : le sac est prêt. [pause]</t>
+          <t>Sous le plancher, le bois du quai tape. Le son grimpe l'escalier, puis la pièce. Dans l'appartement, ça sent le savon et le sel. Une mouette crie contre la vitre. Sur le rebord, un &lt;emphasis&gt;éclat de corde&lt;/emphasis&gt; brille. Il est pâle, raide, et il sent le sel. Le vent du port l'a posé là. Mila ne sait pas à quoi il servira. Son dessin du bateau sèche sur la table. La peinture jaune luit, un peu collante. En bas, le vrai bateau bleu frappe le quai. Je veux le bateau, maintenant ! Mila, tu entends l'eau ? Oui, maman. Il m'attend. On y va, avec le sac. En ce moment, Mila saisit le sac bleu. Le tissu gratte sous ses doigts. La sangle sent le sel, comme la corde. Prends de l'eau, pour le quai. Mila prend la gourde froide. Le goûter sent la pomme, dans son papier. Je mets tout, d'un coup ! Elle pousse gourde, pomme et dessin. Le zip mord le papier du dessin. Le bateau jaune se plie, de travers. Ça reste coincé ! Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>éclat de corde</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,46 +1321,47 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller; emotion=impatience_curieuse; intensite=2; destinataire=enfant; sous_texte=le_bateau_tape_sous_le_plancher; tempo=naturel; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|L'eau du port claque contre le bois.
-narrateur|Une corde mouillée sent le sel.
-narrateur|Les mâts bougent un tout petit peu.
-narrateur|Dans l'appartement au-dessus du quai, ça sent le savon.
-narrateur|Une mouette crie, tout près de la vitre.
-narrateur|Le dessin de Mila sèche près de la fenêtre.
-narrateur|Il sent encore un peu la peinture.
-narrateur|Un bateau bleu attend au bout du quai.
+          <t>narrateur|Sous le plancher, le bois du quai tape.
+narrateur|Le son grimpe l'escalier, puis la pièce.
+narrateur|Dans l'appartement, ça sent le savon et le sel.
+narrateur|Une mouette crie contre la vitre.
+narrateur|Sur le rebord, un éclat de corde brille.
+narrateur|Il est pâle, raide, et il sent le sel.
+narrateur|Le vent du port l'a posé là.
+narrateur|Mila ne sait pas à quoi il servira.
+narrateur|Son dessin du bateau sèche sur la table.
+narrateur|La peinture jaune luit, un peu collante.
+narrateur|En bas, le vrai bateau bleu frappe le quai.
+enfant-f|Je veux le bateau, maintenant !
 maman|Mila, tu entends l'eau ?
 enfant-f|Oui, maman.
-enfant-f|Je veux le bateau.
+enfant-f|Il m'attend.
 maman|On y va, avec le sac.
-narrateur|En ce moment, Mila touche la sangle.
-narrateur|Maman pose le sac bleu près des chaussures.
-narrateur|Le tissu est un peu rêche.
-narrateur|Une chaussure rouge est là.
-narrateur|L'autre n'est pas là.
-enfant-f|Il est bleu, maman.
-maman|Oui, prends de l'eau pour le quai.
-narrateur|Mila prend la gourde.
-narrateur|Elle est froide contre ses doigts.
-narrateur|Elle la met dans le sac.
-narrateur|Le goûter sent la pomme.
-narrateur|Le papier fait un petit bruit.
-maman|Glisse aussi le goûter.
-narrateur|Mila le glisse près de l'eau.
-enfant-f|Et mon doudou ?
-narrateur|Le doudou n'est pas près des chaussures.
-maman|Regarde dans la poche du manteau.
-narrateur|Mila cherche dans la poche.
-narrateur|Le doudou sent le coton.
-enfant-f|Il était caché.
-narrateur|Elle le glisse dans le sac.
-maman|On ouvre ?
-narrateur|Le loquet de la porte résiste.
-enfant-f|Il reste, maman.
-maman|Pousse le petit bouton, tout doux.</t>
+narrateur|En ce moment, Mila saisit le sac bleu.
+narrateur|Le tissu gratte sous ses doigts.
+narrateur|La sangle sent le sel, comme la corde.
+maman|Prends de l'eau, pour le quai.
+narrateur|Mila prend la gourde froide.
+narrateur|Le goûter sent la pomme, dans son papier.
+enfant-f|Je mets tout, d'un coup !
+narrateur|Elle pousse gourde, pomme et dessin.
+narrateur|Le zip mord le papier du dessin.
+narrateur|Le bateau jaune se plie, de travers.
+enfant-f|Ça reste coincé !
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>eau-port,corde,plancher</t>
         </is>
       </c>
     </row>
@@ -1392,12 +1393,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Mila prépare le sac. Où met-elle les affaires ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila prépare le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. Où met-elle les affaires ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Léa prépare le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Que fait-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila prépare le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Où met-elle les affaires ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1460,7 +1461,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1471,7 +1472,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1486,11 +1487,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1501,23 +1502,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1532,17 +1533,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=les_affaires_vont_dans_le_sac; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1575,17 +1576,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mila pousse le bouton du loquet. Le métal est un peu froid. Le loquet cède, tout à coup. Il part. Merci, Mila. Mila ferme le zip du sac. Ça fait zzz. Le sac bleu est fermé. Le sac est prêt ? Oui, maman. Mila pose le sac contre sa jambe. Une chaussure rouge touche le sac. Le dessin jaune attend encore. Tu prends aussi ton dessin ? Oui, pour le bateau. On cherche l'autre chaussure ? Sous le banc.</t>
+          <t>Maman s'accroupit à la même hauteur. Sors le dessin, d'abord. Mila tire le papier coincé. Le zip lâche, petit à petit. Elle pose le dessin à plat, sur la table. L'eau va au fond. Mila range la gourde froide. Le papier de la pomme glisse à côté. Et mon doudou ? Le doudou n'est pas près des chaussures. Regarde dans la poche du manteau. Mila cherche dans la poche. Le doudou sent le coton chaud. Il était caché. Elle le glisse dans le sac. Le zip avance, sans mordre. Il part. Le sac est prêt ? Pas le dessin. Le bateau jaune attend sur la table. Tu prends aussi ton dessin ? Oui, pour le vrai bateau.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila pousse le bouton du loquet. Le métal est un peu froid. Le loquet cède, tout à coup. Il part. Merci, Mila. Mila ferme le zip du sac. Ça fait zzz. Le sac bleu est fermé. Le sac est prêt ? Oui, maman. Mila pose le sac contre sa jambe. Une chaussure rouge touche le sac. Le dessin jaune attend encore. Tu prends aussi ton dessin ? Oui, pour le bateau. On cherche l'autre chaussure ? Sous le banc.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman s'accroupit à la même hauteur. Sors le &lt;emphasis level="moderate"&gt;dessin&lt;/emphasis&gt;, d'abord. Mila tire le papier coincé. Le zip lâche, petit à petit. Elle pose le dessin à plat, sur la table. L'eau va au fond. Mila range la gourde froide. Le papier de la pomme glisse à côté. Et mon doudou ? Le doudou n'est pas près des chaussures. Regarde dans la poche du manteau. Mila cherche dans la poche. Le doudou sent le coton chaud. Il était caché. Elle le glisse dans le sac. Le zip avance, sans mordre. Il part. Le sac est prêt ? Pas le dessin. Le bateau jaune attend sur la table. Tu prends aussi ton dessin ? Oui, pour le vrai bateau.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Léa a mis la gourde, le goûter, le doudou. C'est &lt;emphasis&gt;ce&lt;/emphasis&gt; que maman a dit. [pause]</t>
+          <t>Maman s'accroupit à la même hauteur. Sors le &lt;emphasis&gt;dessin&lt;/emphasis&gt;, d'abord. Mila tire le papier coincé. Le zip lâche, petit à petit. Elle pose le dessin à plat, sur la table. L'eau va au fond. Mila range la gourde froide. Le papier de la pomme glisse à côté. Et mon doudou ? Le doudou n'est pas près des chaussures. Regarde dans la poche du manteau. Mila cherche dans la poche. Le doudou sent le coton chaud. Il était caché. Elle le glisse dans le sac. Le zip avance, sans mordre. Il part. Le sac est prêt ? Pas le dessin. Le bateau jaune attend sur la table. Tu prends aussi ton dessin ? Oui, pour le vrai bateau. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1643,7 +1644,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1666,11 +1667,11 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>ce</t>
+          <t>dessin</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="2" t="n">
         <v>450</v>
@@ -1680,16 +1681,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1714,28 +1715,38 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=une_chose_puis_la_suivante; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Mila pousse le bouton du loquet.
-narrateur|Le métal est un peu froid.
-narrateur|Le loquet cède, tout à coup.
+          <t>narrateur|Maman s'accroupit à la même hauteur.
+maman|Sors le dessin, d'abord.
+narrateur|Mila tire le papier coincé.
+narrateur|Le zip lâche, petit à petit.
+narrateur|Elle pose le dessin à plat, sur la table.
+maman|L'eau va au fond.
+narrateur|Mila range la gourde froide.
+narrateur|Le papier de la pomme glisse à côté.
+enfant-f|Et mon doudou ?
+narrateur|Le doudou n'est pas près des chaussures.
+maman|Regarde dans la poche du manteau.
+narrateur|Mila cherche dans la poche.
+narrateur|Le doudou sent le coton chaud.
+enfant-f|Il était caché.
+narrateur|Elle le glisse dans le sac.
+narrateur|Le zip avance, sans mordre.
 enfant-f|Il part.
-maman|Merci, Mila.
-narrateur|Mila ferme le zip du sac.
-narrateur|Ça fait zzz.
-narrateur|Le sac bleu est fermé.
 maman|Le sac est prêt ?
-enfant-f|Oui, maman.
-narrateur|Mila pose le sac contre sa jambe.
-narrateur|Une chaussure rouge touche le sac.
-narrateur|Le dessin jaune attend encore.
+enfant-f|Pas le dessin.
+narrateur|Le bateau jaune attend sur la table.
 maman|Tu prends aussi ton dessin ?
-enfant-f|Oui, pour le bateau.
-maman|On cherche l'autre chaussure ?
-enfant-f|Sous le banc.</t>
+enfant-f|Oui, pour le vrai bateau.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>zip,tissu</t>
         </is>
       </c>
     </row>
@@ -1762,17 +1773,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On met tes chaussures, maintenant. Mila enfile une chaussure rouge. L'autre est sous le banc. Elle la tire tout doucement. La semelle froide se réchauffe. Tu as fini tes chaussures ? Oui, maman. Mila reprend le sac. Elle tient aussi son dessin. On va vers le quai ? Oui, mon dessin est dans ma main. Elles descendent les marches du port. L'air sent le sel et le bois mouillé. Le bateau bleu tape un peu l'eau. Il est là. Oui, tout près. Mila tient le dessin tout droit. Il ne plie pas. Tu le tiens bien. Une mouette passe tout bas. L'eau claque encore contre le quai.</t>
+          <t>Un souffle entre par la fenêtre. Le dessin glisse vers le rebord. Il va tomber ! Mila veut courir, le papier à la main. Elle veut descendre, sans le sac. Mila refuse de foncer. Attends, je regarde. Sur le rebord, l'éclat de corde tremble. Il penche vers la fenêtre ouverte. C'est le vent ! Le vent vient d'où ? De là, du quai. Mila pousse la fenêtre. Le dessin s'arrête, à plat. Elle glisse l'éclat de corde dans le sac. Puis le dessin, tout à la fin. Le zip ferme, sans mordre. Merci, Mila. On cherche l'autre chaussure ? Sous le banc. Mila enfile une chaussure rouge. L'autre est sous le banc. Elle la tire, sans forcer. Tu as fini tes chaussures ? Oui, maman. On va vers le quai ? Oui, le dessin est dans le sac. Elles descendent les marches du port. L'air sent le sel et le bois mouillé. Le bateau bleu tape un peu l'eau. Il est là. Oui, il est près.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On met tes chaussures, maintenant. Mila enfile une chaussure rouge. L'autre est sous le banc. Elle la tire tout doucement. La semelle froide se réchauffe. Tu as fini tes chaussures ? Oui, maman. Mila reprend le sac. Elle tient aussi son dessin. On va vers le quai ? Oui, mon dessin est dans ma main. Elles descendent les marches du port. L'air sent le sel et le bois mouillé. Le bateau bleu tape un peu l'eau. Il est là. Oui, tout près. Mila tient le dessin tout droit. Il ne plie pas. Tu le tiens bien. Une mouette passe tout bas. L'eau claque encore contre le quai.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un souffle entre par la fenêtre. Le dessin glisse vers le rebord. Il va tomber ! Mila veut courir, le papier à la main. Elle veut descendre, sans le sac. Mila refuse de foncer. Attends, je regarde. Sur le rebord, l'&lt;emphasis level="moderate"&gt;éclat de corde&lt;/emphasis&gt; tremble. Il penche vers la fenêtre ouverte. C'est le vent ! Le vent vient d'où ? De là, du quai. Mila pousse la fenêtre. Le dessin s'arrête, à plat. Elle glisse l'éclat de corde dans le sac. Puis le dessin, tout à la fin. Le zip ferme, sans mordre. Merci, Mila. On cherche l'autre chaussure ? Sous le banc. Mila enfile une chaussure rouge. L'autre est sous le banc. Elle la tire, sans forcer. Tu as fini tes chaussures ? Oui, maman. On va vers le quai ? Oui, le dessin est dans le sac. Elles descendent les marches du port. L'air sent le sel et le bois mouillé. Le bateau bleu tape un peu l'eau. Il est là. Oui, il est près.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman prend le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Elles vont à l'école. [pause]</t>
+          <t>Un souffle entre par la fenêtre. Le dessin glisse vers le rebord. Il va tomber ! Mila veut courir, le papier à la main. Elle veut descendre, sans le sac. Mila refuse de foncer. Attends, je regarde. Sur le rebord, l'&lt;emphasis&gt;éclat de corde&lt;/emphasis&gt; tremble. Il penche vers la fenêtre ouverte. C'est le vent ! Le vent vient d'où ? De là, du quai. Mila pousse la fenêtre. Le dessin s'arrête, à plat. Elle glisse l'éclat de corde dans le sac. Puis le dessin, tout à la fin. Le zip ferme, sans mordre. Merci, Mila. On cherche l'autre chaussure ? Sous le banc. Mila enfile une chaussure rouge. L'autre est sous le banc. Elle la tire, sans forcer. Tu as fini tes chaussures ? Oui, maman. On va vers le quai ? Oui, le dessin est dans le sac. Elles descendent les marches du port. L'air sent le sel et le bois mouillé. Le bateau bleu tape un peu l'eau. Il est là. Oui, il est près. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1819,7 +1830,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1827,10 +1838,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1853,30 +1864,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>éclat de corde</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1885,10 +1896,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1899,30 +1910,50 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=résolution; intention=faire_vivre_la_réussite; emotion=fierté_calme; intensite=2; destinataire=enfant; sous_texte=l_éclat_montre_le_vent; tempo=naturel; sourire=franc; respiration=relâchée</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On met tes chaussures, maintenant.
+          <t>narrateur|Un souffle entre par la fenêtre.
+narrateur|Le dessin glisse vers le rebord.
+enfant-f|Il va tomber !
+narrateur|Mila veut courir, le papier à la main.
+narrateur|Elle veut descendre, sans le sac.
+narrateur|Mila refuse de foncer.
+enfant-f|Attends, je regarde.
+narrateur|Sur le rebord, l'éclat de corde tremble.
+narrateur|Il penche vers la fenêtre ouverte.
+enfant-f|C'est le vent !
+maman|Le vent vient d'où ?
+enfant-f|De là, du quai.
+narrateur|Mila pousse la fenêtre.
+narrateur|Le dessin s'arrête, à plat.
+narrateur|Elle glisse l'éclat de corde dans le sac.
+narrateur|Puis le dessin, tout à la fin.
+narrateur|Le zip ferme, sans mordre.
+maman|Merci, Mila.
+maman|On cherche l'autre chaussure ?
+enfant-f|Sous le banc.
 narrateur|Mila enfile une chaussure rouge.
 narrateur|L'autre est sous le banc.
-narrateur|Elle la tire tout doucement.
-narrateur|La semelle froide se réchauffe.
+narrateur|Elle la tire, sans forcer.
 maman|Tu as fini tes chaussures ?
 enfant-f|Oui, maman.
-narrateur|Mila reprend le sac.
-narrateur|Elle tient aussi son dessin.
 maman|On va vers le quai ?
-enfant-f|Oui, mon dessin est dans ma main.
+enfant-f|Oui, le dessin est dans le sac.
 narrateur|Elles descendent les marches du port.
 narrateur|L'air sent le sel et le bois mouillé.
 narrateur|Le bateau bleu tape un peu l'eau.
 enfant-f|Il est là.
-maman|Oui, tout près.
-narrateur|Mila tient le dessin tout droit.
-enfant-f|Il ne plie pas.
-maman|Tu le tiens bien.
-narrateur|Une mouette passe tout bas.
-narrateur|L'eau claque encore contre le quai.</t>
+maman|Oui, il est près.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>vent,fenetre,marches</t>
         </is>
       </c>
     </row>
@@ -1949,17 +1980,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Mila pose le pied sur le bois du bateau. Le bateau bouge, tout doux. On flotte, maman. Oui, tu es arrivée. Le sac bleu voyage contre sa hanche. Le sel pique un peu les lèvres. Merci pour le sac, Mila. L'eau du port claque encore, tout près.</t>
+          <t>Mila pose le pied sur le bois du bateau. Le bateau bouge, léger. On flotte, maman. Oui, tu es arrivée. Le sac bleu voyage contre sa hanche. Mila ouvre le sac, un peu. L'éclat de corde porte une trace de sel. Le dessin jaune reste plat. Il a voyagé. Comme toi. Le sel pique un peu les lèvres. L'eau du port tape le bois du bateau.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Mila pose le pied sur le bois du bateau. Le bateau bouge, tout doux. On flotte, maman. Oui, tu es arrivée. Le sac bleu voyage contre sa hanche. Le sel pique un peu les lèvres. Merci pour le sac, Mila. L'eau du port claque encore, tout près.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila pose le pied sur le bois du bateau. Le bateau bouge, léger. On flotte, maman. Oui, tu es arrivée. Le sac bleu voyage contre sa hanche. Mila ouvre le sac, un peu. L'&lt;emphasis level="moderate"&gt;éclat de corde&lt;/emphasis&gt; porte une trace de sel. Le dessin jaune reste plat. Il a voyagé. Comme toi. Le sel pique un peu les lèvres. L'eau du port tape le bois du bateau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila pose le pied sur le bois du bateau. Le bateau bouge, léger. On flotte, maman. Oui, tu es arrivée. Le sac bleu voyage contre sa hanche. Mila ouvre le sac, un peu. L'&lt;emphasis&gt;éclat de corde&lt;/emphasis&gt; porte une trace de sel. Le dessin jaune reste plat. Il a voyagé. Comme toi. Le sel pique un peu les lèvres. L'eau du port tape le bois du bateau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2006,18 +2037,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2026,12 +2057,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2040,17 +2071,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de corde</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2059,11 +2094,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2072,31 +2107,44 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_éclat_porte_une_trace_de_sel; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
           <t>narrateur|Mila pose le pied sur le bois du bateau.
-narrateur|Le bateau bouge, tout doux.
+narrateur|Le bateau bouge, léger.
 enfant-f|On flotte, maman.
 maman|Oui, tu es arrivée.
 narrateur|Le sac bleu voyage contre sa hanche.
+narrateur|Mila ouvre le sac, un peu.
+narrateur|L'éclat de corde porte une trace de sel.
+narrateur|Le dessin jaune reste plat.
+enfant-f|Il a voyagé.
+maman|Comme toi.
 narrateur|Le sel pique un peu les lèvres.
-maman|Merci pour le sac, Mila.
-narrateur|L'eau du port claque encore, tout près.</t>
+narrateur|L'eau du port tape le bois du bateau.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>bois,eau,sel</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2209,6 +2257,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): polish ATOM-AUT.AFF.001-04 xlsx
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-04.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-04.xlsx
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sous le plancher, le bois du quai tape. Le son grimpe l'escalier, puis la pièce. Dans l'appartement, ça sent le savon et le sel. Une mouette crie contre la vitre. Sur le rebord, un éclat de corde brille. Il est pâle, raide, et il sent le sel. Le vent du port l'a posé là. Mila ne sait pas à quoi il servira. Son dessin du bateau sèche sur la table. La peinture jaune luit, un peu collante. En bas, le vrai bateau bleu frappe le quai. Je veux le bateau, maintenant ! Mila, tu entends l'eau ? Oui, maman. Il m'attend. On y va, avec le sac. En ce moment, Mila saisit le sac bleu. Le tissu gratte sous ses doigts. La sangle sent le sel, comme la corde. Prends de l'eau, pour le quai. Mila prend la gourde froide. Le goûter sent la pomme, dans son papier. Je mets tout, d'un coup ! Elle pousse gourde, pomme et dessin. Le zip mord le papier du dessin. Le bateau jaune se plie, de travers. Ça reste coincé ! Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent.</t>
+          <t>Sous le plancher, le bois du quai tape. Le son grimpe l'escalier, puis la pièce. Dans l'appartement, ça sent le savon et le sel. Une mouette crie contre la vitre. Sur le rebord, un éclat de corde brille. Il est pâle, raide, et il sent le sel. Le vent du port l'a posé là. Mila le touche du doigt, puis le laisse. Son dessin du bateau sèche sur la table. La peinture jaune luit, un peu collante. En bas, le vrai bateau bleu frappe le quai. Je veux le bateau, maintenant ! Mila, tu entends l'eau ? Oui, maman. Il m'attend. On y va, avec le sac. En ce moment, Mila saisit le sac bleu. Le tissu gratte sous ses doigts. La sangle sent le sel, comme la corde. Prends de l'eau, pour le quai. Mila prend la gourde froide. Le goûter sent la pomme, dans son papier. Je mets tout, d'un coup ! Elle pousse gourde, pomme et dessin. Le zip mord le papier du dessin. Le bateau jaune se plie, de travers. Ça reste coincé ! Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sous le plancher, le bois du quai tape. Le son grimpe l'escalier, puis la pièce. Dans l'appartement, ça sent le savon et le sel. Une mouette crie contre la vitre. Sur le rebord, un &lt;emphasis level="moderate"&gt;éclat de corde&lt;/emphasis&gt; brille. Il est pâle, raide, et il sent le sel. Le vent du port l'a posé là. Mila ne sait pas à quoi il servira. Son dessin du bateau sèche sur la table. La peinture jaune luit, un peu collante. En bas, le vrai bateau bleu frappe le quai. Je veux le bateau, maintenant ! Mila, tu entends l'eau ? Oui, maman. Il m'attend. On y va, avec le sac. En ce moment, Mila saisit le sac bleu. Le tissu gratte sous ses doigts. La sangle sent le sel, comme la corde. Prends de l'eau, pour le quai. Mila prend la gourde froide. Le goûter sent la pomme, dans son papier. Je mets tout, d'un coup ! Elle pousse gourde, pomme et dessin. Le zip mord le papier du dessin. Le bateau jaune se plie, de travers. Ça reste coincé ! Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sous le plancher, le bois du quai tape. Le son grimpe l'escalier, puis la pièce. Dans l'appartement, ça sent le savon et le sel. Une mouette crie contre la vitre. Sur le rebord, un &lt;emphasis level="moderate"&gt;éclat de corde&lt;/emphasis&gt; brille. Il est pâle, raide, et il sent le sel. Le vent du port l'a posé là. Mila le touche du doigt, puis le laisse. Son dessin du bateau sèche sur la table. La peinture jaune luit, un peu collante. En bas, le vrai bateau bleu frappe le quai. Je veux le bateau, maintenant ! Mila, tu entends l'eau ? Oui, maman. Il m'attend. On y va, avec le sac. En ce moment, Mila saisit le sac bleu. Le tissu gratte sous ses doigts. La sangle sent le sel, comme la corde. Prends de l'eau, pour le quai. Mila prend la gourde froide. Le goûter sent la pomme, dans son papier. Je mets tout, d'un coup ! Elle pousse gourde, pomme et dessin. Le zip mord le papier du dessin. Le bateau jaune se plie, de travers. Ça reste coincé ! Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Sous le plancher, le bois du quai tape. Le son grimpe l'escalier, puis la pièce. Dans l'appartement, ça sent le savon et le sel. Une mouette crie contre la vitre. Sur le rebord, un &lt;emphasis&gt;éclat de corde&lt;/emphasis&gt; brille. Il est pâle, raide, et il sent le sel. Le vent du port l'a posé là. Mila ne sait pas à quoi il servira. Son dessin du bateau sèche sur la table. La peinture jaune luit, un peu collante. En bas, le vrai bateau bleu frappe le quai. Je veux le bateau, maintenant ! Mila, tu entends l'eau ? Oui, maman. Il m'attend. On y va, avec le sac. En ce moment, Mila saisit le sac bleu. Le tissu gratte sous ses doigts. La sangle sent le sel, comme la corde. Prends de l'eau, pour le quai. Mila prend la gourde froide. Le goûter sent la pomme, dans son papier. Je mets tout, d'un coup ! Elle pousse gourde, pomme et dessin. Le zip mord le papier du dessin. Le bateau jaune se plie, de travers. Ça reste coincé ! Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. [pause]</t>
+          <t>Sous le plancher, le bois du quai tape. Le son grimpe l'escalier, puis la pièce. Dans l'appartement, ça sent le savon et le sel. Une mouette crie contre la vitre. Sur le rebord, un &lt;emphasis&gt;éclat de corde&lt;/emphasis&gt; brille. Il est pâle, raide, et il sent le sel. Le vent du port l'a posé là. Mila le touche du doigt, puis le laisse. Son dessin du bateau sèche sur la table. La peinture jaune luit, un peu collante. En bas, le vrai bateau bleu frappe le quai. Je veux le bateau, maintenant ! Mila, tu entends l'eau ? Oui, maman. Il m'attend. On y va, avec le sac. En ce moment, Mila saisit le sac bleu. Le tissu gratte sous ses doigts. La sangle sent le sel, comme la corde. Prends de l'eau, pour le quai. Mila prend la gourde froide. Le goûter sent la pomme, dans son papier. Je mets tout, d'un coup ! Elle pousse gourde, pomme et dessin. Le zip mord le papier du dessin. Le bateau jaune se plie, de travers. Ça reste coincé ! Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1335,7 +1335,7 @@
 narrateur|Sur le rebord, un éclat de corde brille.
 narrateur|Il est pâle, raide, et il sent le sel.
 narrateur|Le vent du port l'a posé là.
-narrateur|Mila ne sait pas à quoi il servira.
+narrateur|Mila le touche du doigt, puis le laisse.
 narrateur|Son dessin du bateau sèche sur la table.
 narrateur|La peinture jaune luit, un peu collante.
 narrateur|En bas, le vrai bateau bleu frappe le quai.
@@ -1773,17 +1773,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Un souffle entre par la fenêtre. Le dessin glisse vers le rebord. Il va tomber ! Mila veut courir, le papier à la main. Elle veut descendre, sans le sac. Mila refuse de foncer. Attends, je regarde. Sur le rebord, l'éclat de corde tremble. Il penche vers la fenêtre ouverte. C'est le vent ! Le vent vient d'où ? De là, du quai. Mila pousse la fenêtre. Le dessin s'arrête, à plat. Elle glisse l'éclat de corde dans le sac. Puis le dessin, tout à la fin. Le zip ferme, sans mordre. Merci, Mila. On cherche l'autre chaussure ? Sous le banc. Mila enfile une chaussure rouge. L'autre est sous le banc. Elle la tire, sans forcer. Tu as fini tes chaussures ? Oui, maman. On va vers le quai ? Oui, le dessin est dans le sac. Elles descendent les marches du port. L'air sent le sel et le bois mouillé. Le bateau bleu tape un peu l'eau. Il est là. Oui, il est près.</t>
+          <t>Un souffle entre par la fenêtre. Le dessin glisse vers le rebord. Il va tomber ! Mila veut courir, le papier à la main. Elle veut descendre, sans le sac. Mila refuse de foncer. Attends, je regarde. Sur le rebord, l'éclat de corde tremble. Il penche vers la fenêtre ouverte. C'est le vent ! Le vent vient d'où ? De là, du quai. Mila pousse la fenêtre. Le dessin s'arrête, à plat. Elle glisse l'éclat de corde dans le sac. Puis le dessin, à la fin. Le zip glisse jusqu'au bout. Merci, Mila. On va vers le quai ? Oui, le dessin est dans le sac. Mila passe la sangle sur l'épaule. Elles descendent les marches du port. L'air sent le sel et le bois mouillé. Une corde mouillée frappe un anneau. Le bateau bleu tape l'eau. Il est là. Oui, il est près.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un souffle entre par la fenêtre. Le dessin glisse vers le rebord. Il va tomber ! Mila veut courir, le papier à la main. Elle veut descendre, sans le sac. Mila refuse de foncer. Attends, je regarde. Sur le rebord, l'&lt;emphasis level="moderate"&gt;éclat de corde&lt;/emphasis&gt; tremble. Il penche vers la fenêtre ouverte. C'est le vent ! Le vent vient d'où ? De là, du quai. Mila pousse la fenêtre. Le dessin s'arrête, à plat. Elle glisse l'éclat de corde dans le sac. Puis le dessin, tout à la fin. Le zip ferme, sans mordre. Merci, Mila. On cherche l'autre chaussure ? Sous le banc. Mila enfile une chaussure rouge. L'autre est sous le banc. Elle la tire, sans forcer. Tu as fini tes chaussures ? Oui, maman. On va vers le quai ? Oui, le dessin est dans le sac. Elles descendent les marches du port. L'air sent le sel et le bois mouillé. Le bateau bleu tape un peu l'eau. Il est là. Oui, il est près.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un souffle entre par la fenêtre. Le dessin glisse vers le rebord. Il va tomber ! Mila veut courir, le papier à la main. Elle veut descendre, sans le sac. Mila refuse de foncer. Attends, je regarde. Sur le rebord, l'&lt;emphasis level="moderate"&gt;éclat de corde&lt;/emphasis&gt; tremble. Il penche vers la fenêtre ouverte. C'est le vent ! Le vent vient d'où ? De là, du quai. Mila pousse la fenêtre. Le dessin s'arrête, à plat. Elle glisse l'éclat de corde dans le sac. Puis le dessin, à la fin. Le zip glisse jusqu'au bout. Merci, Mila. On va vers le quai ? Oui, le dessin est dans le sac. Mila passe la sangle sur l'épaule. Elles descendent les marches du port. L'air sent le sel et le bois mouillé. Une corde mouillée frappe un anneau. Le bateau bleu tape l'eau. Il est là. Oui, il est près.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Un souffle entre par la fenêtre. Le dessin glisse vers le rebord. Il va tomber ! Mila veut courir, le papier à la main. Elle veut descendre, sans le sac. Mila refuse de foncer. Attends, je regarde. Sur le rebord, l'&lt;emphasis&gt;éclat de corde&lt;/emphasis&gt; tremble. Il penche vers la fenêtre ouverte. C'est le vent ! Le vent vient d'où ? De là, du quai. Mila pousse la fenêtre. Le dessin s'arrête, à plat. Elle glisse l'éclat de corde dans le sac. Puis le dessin, tout à la fin. Le zip ferme, sans mordre. Merci, Mila. On cherche l'autre chaussure ? Sous le banc. Mila enfile une chaussure rouge. L'autre est sous le banc. Elle la tire, sans forcer. Tu as fini tes chaussures ? Oui, maman. On va vers le quai ? Oui, le dessin est dans le sac. Elles descendent les marches du port. L'air sent le sel et le bois mouillé. Le bateau bleu tape un peu l'eau. Il est là. Oui, il est près. [pause]</t>
+          <t>Un souffle entre par la fenêtre. Le dessin glisse vers le rebord. Il va tomber ! Mila veut courir, le papier à la main. Elle veut descendre, sans le sac. Mila refuse de foncer. Attends, je regarde. Sur le rebord, l'&lt;emphasis&gt;éclat de corde&lt;/emphasis&gt; tremble. Il penche vers la fenêtre ouverte. C'est le vent ! Le vent vient d'où ? De là, du quai. Mila pousse la fenêtre. Le dessin s'arrête, à plat. Elle glisse l'éclat de corde dans le sac. Puis le dessin, à la fin. Le zip glisse jusqu'au bout. Merci, Mila. On va vers le quai ? Oui, le dessin est dans le sac. Mila passe la sangle sur l'épaule. Elles descendent les marches du port. L'air sent le sel et le bois mouillé. Une corde mouillée frappe un anneau. Le bateau bleu tape l'eau. Il est là. Oui, il est près. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="AV5" s="2" t="inlineStr">
         <is>
-          <t>arc=résolution; intention=faire_vivre_la_réussite; emotion=fierté_calme; intensite=2; destinataire=enfant; sous_texte=l_éclat_montre_le_vent; tempo=naturel; sourire=franc; respiration=relâchée</t>
+          <t>arc=résolution; intention=faire_vivre_la_réussite; emotion=fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_l_éclat_dit_le_vent; tempo=naturel; sourire=franc; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW5" t="inlineStr">
@@ -1932,21 +1932,16 @@
 narrateur|Mila pousse la fenêtre.
 narrateur|Le dessin s'arrête, à plat.
 narrateur|Elle glisse l'éclat de corde dans le sac.
-narrateur|Puis le dessin, tout à la fin.
-narrateur|Le zip ferme, sans mordre.
+narrateur|Puis le dessin, à la fin.
+narrateur|Le zip glisse jusqu'au bout.
 maman|Merci, Mila.
-maman|On cherche l'autre chaussure ?
-enfant-f|Sous le banc.
-narrateur|Mila enfile une chaussure rouge.
-narrateur|L'autre est sous le banc.
-narrateur|Elle la tire, sans forcer.
-maman|Tu as fini tes chaussures ?
-enfant-f|Oui, maman.
 maman|On va vers le quai ?
 enfant-f|Oui, le dessin est dans le sac.
+narrateur|Mila passe la sangle sur l'épaule.
 narrateur|Elles descendent les marches du port.
 narrateur|L'air sent le sel et le bois mouillé.
-narrateur|Le bateau bleu tape un peu l'eau.
+narrateur|Une corde mouillée frappe un anneau.
+narrateur|Le bateau bleu tape l'eau.
 enfant-f|Il est là.
 maman|Oui, il est près.</t>
         </is>
@@ -1980,17 +1975,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Mila pose le pied sur le bois du bateau. Le bateau bouge, léger. On flotte, maman. Oui, tu es arrivée. Le sac bleu voyage contre sa hanche. Mila ouvre le sac, un peu. L'éclat de corde porte une trace de sel. Le dessin jaune reste plat. Il a voyagé. Comme toi. Le sel pique un peu les lèvres. L'eau du port tape le bois du bateau.</t>
+          <t>Mila pose le pied sur le bois du bateau. Le bateau bouge, léger. On flotte, maman. Oui, tu es arrivée. Le sac bleu voyage contre sa hanche. Mila ouvre le sac. L'éclat de corde porte une trace de sel. Le dessin jaune reste plat. Il a voyagé. Comme toi. Le sel pique un peu les lèvres. L'eau du port tape le bois du bateau.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila pose le pied sur le bois du bateau. Le bateau bouge, léger. On flotte, maman. Oui, tu es arrivée. Le sac bleu voyage contre sa hanche. Mila ouvre le sac, un peu. L'&lt;emphasis level="moderate"&gt;éclat de corde&lt;/emphasis&gt; porte une trace de sel. Le dessin jaune reste plat. Il a voyagé. Comme toi. Le sel pique un peu les lèvres. L'eau du port tape le bois du bateau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Mila pose le pied sur le bois du bateau. Le bateau bouge, léger. On flotte, maman. Oui, tu es arrivée. Le sac bleu voyage contre sa hanche. Mila ouvre le sac. L'&lt;emphasis level="moderate"&gt;éclat de corde&lt;/emphasis&gt; porte une trace de sel. Le dessin jaune reste plat. Il a voyagé. Comme toi. Le sel pique un peu les lèvres. L'eau du port tape le bois du bateau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila pose le pied sur le bois du bateau. Le bateau bouge, léger. On flotte, maman. Oui, tu es arrivée. Le sac bleu voyage contre sa hanche. Mila ouvre le sac, un peu. L'&lt;emphasis&gt;éclat de corde&lt;/emphasis&gt; porte une trace de sel. Le dessin jaune reste plat. Il a voyagé. Comme toi. Le sel pique un peu les lèvres. L'eau du port tape le bois du bateau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Mila pose le pied sur le bois du bateau. Le bateau bouge, léger. On flotte, maman. Oui, tu es arrivée. Le sac bleu voyage contre sa hanche. Mila ouvre le sac. L'&lt;emphasis&gt;éclat de corde&lt;/emphasis&gt; porte une trace de sel. Le dessin jaune reste plat. Il a voyagé. Comme toi. Le sel pique un peu les lèvres. L'eau du port tape le bois du bateau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2133,7 +2128,7 @@
 enfant-f|On flotte, maman.
 maman|Oui, tu es arrivée.
 narrateur|Le sac bleu voyage contre sa hanche.
-narrateur|Mila ouvre le sac, un peu.
+narrateur|Mila ouvre le sac.
 narrateur|L'éclat de corde porte une trace de sel.
 narrateur|Le dessin jaune reste plat.
 enfant-f|Il a voyagé.
@@ -2165,7 +2160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2264,6 +2259,13 @@
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>